<commit_message>
Added all recent changes
</commit_message>
<xml_diff>
--- a/backend/Childsurvey.xlsx
+++ b/backend/Childsurvey.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W523"/>
+  <dimension ref="A1:W530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32689,6 +32689,378 @@
       <c r="V523" t="inlineStr"/>
       <c r="W523" t="inlineStr"/>
     </row>
+    <row r="524">
+      <c r="A524" t="inlineStr"/>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Divyansh Bafila</t>
+        </is>
+      </c>
+      <c r="C524" t="n">
+        <v>14</v>
+      </c>
+      <c r="D524" t="inlineStr"/>
+      <c r="E524" t="n">
+        <v>11</v>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Financial </t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lack of Confidence
+</t>
+        </is>
+      </c>
+      <c r="I524" t="n">
+        <v>5</v>
+      </c>
+      <c r="J524" t="n">
+        <v>700</v>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>Army</t>
+        </is>
+      </c>
+      <c r="L524" t="inlineStr"/>
+      <c r="M524" t="inlineStr"/>
+      <c r="N524" t="inlineStr"/>
+      <c r="O524" t="inlineStr"/>
+      <c r="P524" t="inlineStr"/>
+      <c r="Q524" t="inlineStr"/>
+      <c r="R524" t="inlineStr"/>
+      <c r="S524" t="inlineStr"/>
+      <c r="T524" t="inlineStr"/>
+      <c r="U524" t="inlineStr"/>
+      <c r="V524" t="inlineStr"/>
+      <c r="W524" t="inlineStr"/>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr"/>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Ayush Lavania</t>
+        </is>
+      </c>
+      <c r="C525" t="n">
+        <v>5</v>
+      </c>
+      <c r="D525" t="inlineStr"/>
+      <c r="E525" t="n">
+        <v>12</v>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I525" t="n">
+        <v>5</v>
+      </c>
+      <c r="J525" t="n">
+        <v>700</v>
+      </c>
+      <c r="K525" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
+      </c>
+      <c r="L525" t="inlineStr"/>
+      <c r="M525" t="inlineStr"/>
+      <c r="N525" t="inlineStr"/>
+      <c r="O525" t="inlineStr"/>
+      <c r="P525" t="inlineStr"/>
+      <c r="Q525" t="inlineStr"/>
+      <c r="R525" t="inlineStr"/>
+      <c r="S525" t="inlineStr"/>
+      <c r="T525" t="inlineStr"/>
+      <c r="U525" t="inlineStr"/>
+      <c r="V525" t="inlineStr"/>
+      <c r="W525" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr"/>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Ayush Lavania</t>
+        </is>
+      </c>
+      <c r="C526" t="n">
+        <v>14</v>
+      </c>
+      <c r="D526" t="inlineStr"/>
+      <c r="E526" t="n">
+        <v>5</v>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>aggresive</t>
+        </is>
+      </c>
+      <c r="I526" t="n">
+        <v>5</v>
+      </c>
+      <c r="J526" t="n">
+        <v>700</v>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>teacher</t>
+        </is>
+      </c>
+      <c r="L526" t="inlineStr"/>
+      <c r="M526" t="inlineStr"/>
+      <c r="N526" t="inlineStr"/>
+      <c r="O526" t="inlineStr"/>
+      <c r="P526" t="inlineStr"/>
+      <c r="Q526" t="inlineStr"/>
+      <c r="R526" t="inlineStr"/>
+      <c r="S526" t="inlineStr"/>
+      <c r="T526" t="inlineStr"/>
+      <c r="U526" t="inlineStr"/>
+      <c r="V526" t="inlineStr"/>
+      <c r="W526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr"/>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Ayush Lavania</t>
+        </is>
+      </c>
+      <c r="C527" t="n">
+        <v>9</v>
+      </c>
+      <c r="D527" t="inlineStr"/>
+      <c r="E527" t="n">
+        <v>3</v>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Middle Class</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>lack of confidence</t>
+        </is>
+      </c>
+      <c r="I527" t="n">
+        <v>8</v>
+      </c>
+      <c r="J527" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K527" t="inlineStr">
+        <is>
+          <t>Army</t>
+        </is>
+      </c>
+      <c r="L527" t="inlineStr"/>
+      <c r="M527" t="inlineStr"/>
+      <c r="N527" t="inlineStr"/>
+      <c r="O527" t="inlineStr"/>
+      <c r="P527" t="inlineStr"/>
+      <c r="Q527" t="inlineStr"/>
+      <c r="R527" t="inlineStr"/>
+      <c r="S527" t="inlineStr"/>
+      <c r="T527" t="inlineStr"/>
+      <c r="U527" t="inlineStr"/>
+      <c r="V527" t="inlineStr"/>
+      <c r="W527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr"/>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Ayush Lavania</t>
+        </is>
+      </c>
+      <c r="C528" t="n">
+        <v>9</v>
+      </c>
+      <c r="D528" t="inlineStr"/>
+      <c r="E528" t="n">
+        <v>3</v>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>Middle Class</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>lack of confidence</t>
+        </is>
+      </c>
+      <c r="I528" t="n">
+        <v>8</v>
+      </c>
+      <c r="J528" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>Army</t>
+        </is>
+      </c>
+      <c r="L528" t="inlineStr"/>
+      <c r="M528" t="inlineStr"/>
+      <c r="N528" t="inlineStr"/>
+      <c r="O528" t="inlineStr"/>
+      <c r="P528" t="inlineStr"/>
+      <c r="Q528" t="inlineStr"/>
+      <c r="R528" t="inlineStr"/>
+      <c r="S528" t="inlineStr"/>
+      <c r="T528" t="inlineStr"/>
+      <c r="U528" t="inlineStr"/>
+      <c r="V528" t="inlineStr"/>
+      <c r="W528" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr"/>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Ayush Lavania</t>
+        </is>
+      </c>
+      <c r="C529" t="n">
+        <v>12</v>
+      </c>
+      <c r="D529" t="inlineStr"/>
+      <c r="E529" t="n">
+        <v>7</v>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Financial </t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Aggresive</t>
+        </is>
+      </c>
+      <c r="I529" t="n">
+        <v>2</v>
+      </c>
+      <c r="J529" t="n">
+        <v>500</v>
+      </c>
+      <c r="K529" t="inlineStr">
+        <is>
+          <t>Army</t>
+        </is>
+      </c>
+      <c r="L529" t="inlineStr"/>
+      <c r="M529" t="inlineStr"/>
+      <c r="N529" t="inlineStr"/>
+      <c r="O529" t="inlineStr"/>
+      <c r="P529" t="inlineStr"/>
+      <c r="Q529" t="inlineStr"/>
+      <c r="R529" t="inlineStr"/>
+      <c r="S529" t="inlineStr"/>
+      <c r="T529" t="inlineStr"/>
+      <c r="U529" t="inlineStr"/>
+      <c r="V529" t="inlineStr"/>
+      <c r="W529" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr"/>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Ayush Lavania</t>
+        </is>
+      </c>
+      <c r="C530" t="n">
+        <v>15</v>
+      </c>
+      <c r="D530" t="inlineStr"/>
+      <c r="E530" t="n">
+        <v>10</v>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>Middle Class</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>lack of confidence</t>
+        </is>
+      </c>
+      <c r="I530" t="n">
+        <v>6</v>
+      </c>
+      <c r="J530" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>Army</t>
+        </is>
+      </c>
+      <c r="L530" t="inlineStr"/>
+      <c r="M530" t="inlineStr"/>
+      <c r="N530" t="inlineStr"/>
+      <c r="O530" t="inlineStr"/>
+      <c r="P530" t="inlineStr"/>
+      <c r="Q530" t="inlineStr"/>
+      <c r="R530" t="inlineStr"/>
+      <c r="S530" t="inlineStr"/>
+      <c r="T530" t="inlineStr"/>
+      <c r="U530" t="inlineStr"/>
+      <c r="V530" t="inlineStr"/>
+      <c r="W530" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>